<commit_message>
Updated QADemo test scripts, POM classes and  screenshots
</commit_message>
<xml_diff>
--- a/ecom.BITM.QADemo/src/test/resources/QADemo/QADemo.xlsx
+++ b/ecom.BITM.QADemo/src/test/resources/QADemo/QADemo.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4505"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\eclipse-workspace\ecom.BITM.QADemo\src\test\resources\QADemo\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F36D118-ED71-4149-816C-7B14762217B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="2450" windowWidth="11630" windowHeight="2570" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -18,7 +12,8 @@
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
+  <oleSize ref="A1:H8"/>
 </workbook>
 </file>
 
@@ -72,31 +67,9 @@
     <t>Confirm Password</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color indexed="15"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>ammu</t>
-    </r>
-  </si>
-  <si>
     <t>98978</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color indexed="15"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Ammu@123</t>
-    </r>
-  </si>
-  <si>
     <t>standard_user</t>
   </si>
   <si>
@@ -133,15 +106,6 @@
     <t>Name on Card</t>
   </si>
   <si>
-    <t>Ammu</t>
-  </si>
-  <si>
-    <t>Reddy</t>
-  </si>
-  <si>
-    <t>Gandhinagar</t>
-  </si>
-  <si>
     <t>4242 4242 4242 4242</t>
   </si>
   <si>
@@ -151,9 +115,6 @@
     <t>123</t>
   </si>
   <si>
-    <t>Ammuu</t>
-  </si>
-  <si>
     <t xml:space="preserve">      </t>
   </si>
   <si>
@@ -170,13 +131,31 @@
   </si>
   <si>
     <t xml:space="preserve">          </t>
+  </si>
+  <si>
+    <t>Indu</t>
+  </si>
+  <si>
+    <t>Indu@1234</t>
+  </si>
+  <si>
+    <t>Hanu</t>
+  </si>
+  <si>
+    <t>vvnagar</t>
+  </si>
+  <si>
+    <t>Induu</t>
+  </si>
+  <si>
+    <t>Indu003</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -206,7 +185,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color indexed="15"/>
+      <color theme="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -408,10 +387,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -458,12 +441,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="10" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1591,12 +1576,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2" style="4" customWidth="1"/>
     <col min="2" max="4" width="30.453125" style="4" customWidth="1"/>
@@ -1604,51 +1589,51 @@
     <col min="7" max="16384" width="10" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="13.5" customHeight="1">
       <c r="A1" s="5"/>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="7"/>
     </row>
-    <row r="2" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="13.5" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="0" hidden="1" customHeight="1">
       <c r="A3" s="8"/>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="13.5" customHeight="1">
       <c r="A4" s="8"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="13.5" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="10"/>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="13.5" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="10"/>
     </row>
-    <row r="7" spans="1:5" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" ht="18.5">
       <c r="A7" s="8"/>
       <c r="B7" s="11" t="s">
         <v>1</v>
@@ -1661,14 +1646,14 @@
       </c>
       <c r="E7" s="10"/>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="13.5" customHeight="1">
       <c r="A8" s="8"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="10"/>
     </row>
-    <row r="9" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="15.5">
       <c r="A9" s="8"/>
       <c r="B9" s="12" t="s">
         <v>5</v>
@@ -1677,7 +1662,7 @@
       <c r="D9" s="13"/>
       <c r="E9" s="10"/>
     </row>
-    <row r="10" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="15.5">
       <c r="A10" s="8"/>
       <c r="B10" s="14"/>
       <c r="C10" s="15" t="s">
@@ -1688,7 +1673,7 @@
       </c>
       <c r="E10" s="10"/>
     </row>
-    <row r="11" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="13" customHeight="1">
       <c r="A11" s="8"/>
       <c r="B11" s="1" t="s">
         <v>5</v>
@@ -1697,7 +1682,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="10"/>
     </row>
-    <row r="12" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="13" customHeight="1">
       <c r="A12" s="8"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
@@ -1708,7 +1693,7 @@
       </c>
       <c r="E12" s="10"/>
     </row>
-    <row r="13" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="13" customHeight="1">
       <c r="A13" s="8"/>
       <c r="B13" s="1" t="s">
         <v>7</v>
@@ -1717,7 +1702,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="10"/>
     </row>
-    <row r="14" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="13" customHeight="1">
       <c r="A14" s="17"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
@@ -1728,7 +1713,7 @@
       </c>
       <c r="E14" s="18"/>
     </row>
-    <row r="15" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="13" customHeight="1">
       <c r="A15" s="5"/>
       <c r="B15" s="1" t="s">
         <v>8</v>
@@ -1737,7 +1722,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="7"/>
     </row>
-    <row r="16" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="13" customHeight="1">
       <c r="A16" s="17"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
@@ -1753,14 +1738,10 @@
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D10" location="'Export Summary'!R1C1" display="Export Summary" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="D10" location="'Sheet1'!R1C1" display="Sheet1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="D12" location="'Sheet1'!R1C1" display="Sheet1" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="D14" location="'Sheet2'!R1C1" display="Sheet2" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="D16" location="'Sheet3'!R1C1" display="Sheet3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="D12" location="'Sheet1'!R1C1" display="Sheet1" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="D14" location="'Sheet2'!R1C1" display="Sheet2" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="D16" location="'Sheet3'!R1C1" display="Sheet3" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D10" location="'Sheet1'!R1C1" display="Sheet1"/>
+    <hyperlink ref="D12" location="'Sheet1'!R1C1" display="Sheet1"/>
+    <hyperlink ref="D14" location="'Sheet2'!R1C1" display="Sheet2"/>
+    <hyperlink ref="D16" location="'Sheet3'!R1C1" display="Sheet3"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>
@@ -1771,9 +1752,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17.36328125" style="4" customWidth="1"/>
     <col min="2" max="2" width="14.1796875" style="4" customWidth="1"/>
@@ -1783,7 +1764,7 @@
     <col min="7" max="16384" width="8.81640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="13.5" customHeight="1">
       <c r="A1" s="19" t="s">
         <v>9</v>
       </c>
@@ -1798,79 +1779,79 @@
       </c>
       <c r="E1" s="21"/>
     </row>
-    <row r="2" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:5" ht="13.5" customHeight="1">
+      <c r="A2" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="C2" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="22"/>
+    </row>
+    <row r="3" spans="1:5" ht="13.5" customHeight="1">
+      <c r="A3" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="B3" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="22"/>
-    </row>
-    <row r="3" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="19" t="s">
+      <c r="C3" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>18</v>
-      </c>
       <c r="D3" s="19" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E3" s="22"/>
     </row>
-    <row r="4" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="13.5" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="13.5" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="10"/>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="13.5" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="10"/>
     </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="13.5" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="10"/>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="13.5" customHeight="1">
       <c r="A8" s="8"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="10"/>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="13.5" customHeight="1">
       <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="10"/>
     </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="13.5" customHeight="1">
       <c r="A10" s="17"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>
@@ -1879,9 +1860,9 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="C2" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="D2" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="A2" r:id="rId1" display="Indu03@example.com"/>
+    <hyperlink ref="C2" r:id="rId2"/>
+    <hyperlink ref="D2" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1892,9 +1873,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="13.36328125" style="4" customWidth="1"/>
     <col min="2" max="2" width="11.1796875" style="4" customWidth="1"/>
@@ -1902,9 +1883,9 @@
     <col min="7" max="16384" width="8.81640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="13.5" customHeight="1">
       <c r="A1" s="19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B1" s="19" t="s">
         <v>11</v>
@@ -1913,67 +1894,67 @@
       <c r="D1" s="6"/>
       <c r="E1" s="7"/>
     </row>
-    <row r="2" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="13.5" customHeight="1">
       <c r="A2" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>16</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>18</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="13.5" customHeight="1">
       <c r="A3" s="24"/>
       <c r="B3" s="25"/>
       <c r="C3" s="8"/>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="13.5" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="13.5" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="10"/>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="13.5" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="10"/>
     </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="13.5" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="10"/>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="13.5" customHeight="1">
       <c r="A8" s="8"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="10"/>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="13.5" customHeight="1">
       <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="10"/>
     </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="13.5" customHeight="1">
       <c r="A10" s="17"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>
@@ -1990,9 +1971,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.36328125" style="4" customWidth="1"/>
     <col min="2" max="2" width="13.26953125" style="4" customWidth="1"/>
@@ -2007,94 +1988,94 @@
     <col min="11" max="16384" width="8.81640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="13.5" customHeight="1">
       <c r="A1" s="19" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B1" s="19" t="s">
         <v>11</v>
       </c>
       <c r="C1" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="F1" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="G1" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="H1" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="I1" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="19" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="13.5" customHeight="1">
+      <c r="A2" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="G2" s="19" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="19" t="s">
+      <c r="H2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="13.5" customHeight="1">
+      <c r="A3" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="19" t="s">
+      <c r="C3" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="D3" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="E3" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="19" t="s">
+      <c r="F3" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="G3" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I3" s="25" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="H3" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" s="25" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="13.5" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -2105,7 +2086,7 @@
       <c r="H4" s="6"/>
       <c r="I4" s="7"/>
     </row>
-    <row r="5" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="13.5" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -2116,7 +2097,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="13.5" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -2127,7 +2108,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="13.5" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -2138,7 +2119,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="10"/>
     </row>
-    <row r="8" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="13.5" customHeight="1">
       <c r="A8" s="8"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -2148,7 +2129,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="10"/>
     </row>
-    <row r="9" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="13.5" customHeight="1">
       <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -2159,7 +2140,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="13.5" customHeight="1">
       <c r="A10" s="17"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>

</xml_diff>